<commit_message>
fix template inventory product
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ImportInventoryProductTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ImportInventoryProductTemplate.xlsx
@@ -139,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -149,6 +149,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -433,7 +439,9 @@
   <dimension ref="A1:Z1"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="17" width="24" style="1" customWidth="1"/>
+    <col min="1" max="5" width="24" style="1" customWidth="1"/>
+    <col min="6" max="6" width="24" style="5" customWidth="1"/>
+    <col min="7" max="17" width="24" style="1" customWidth="1"/>
     <col min="18" max="18" width="10" style="1" customWidth="1"/>
     <col min="19" max="19" width="11" style="1" customWidth="1"/>
     <col min="20" max="20" width="11.7109375" style="1" customWidth="1"/>
@@ -456,7 +464,7 @@
       <c r="E1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="G1" s="3" t="s">

</xml_diff>

<commit_message>
inventory ins 30 day
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ImportInventoryProductTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ImportInventoryProductTemplate.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Số lớp</t>
   </si>
@@ -70,12 +70,6 @@
   </si>
   <si>
     <t>Đội</t>
-  </si>
-  <si>
-    <t>Số tấm thành phẩm OK</t>
-  </si>
-  <si>
-    <t>KTNQ 30 NGAY</t>
   </si>
 </sst>
 </file>
@@ -476,19 +470,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z1"/>
+  <dimension ref="A1:X1"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="5" width="24" style="1" customWidth="1"/>
     <col min="6" max="6" width="24" style="4" customWidth="1"/>
     <col min="7" max="17" width="24" style="1" customWidth="1"/>
-    <col min="18" max="18" width="27.5703125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="23.28515625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="11.7109375" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="9.140625" style="1"/>
+    <col min="18" max="18" width="11.7109375" style="1" customWidth="1"/>
+    <col min="19" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="2" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" s="2" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>6</v>
       </c>
@@ -540,19 +532,13 @@
       <c r="Q1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="5"/>
+      <c r="R1" s="5"/>
+      <c r="S1" s="3"/>
+      <c r="T1" s="3"/>
       <c r="U1" s="3"/>
       <c r="V1" s="3"/>
       <c r="W1" s="3"/>
       <c r="X1" s="3"/>
-      <c r="Y1" s="3"/>
-      <c r="Z1" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>